<commit_message>
fix(studio): bundle offline Tailwind CSS and CodeMirror assets to fix slow loading and missing styles
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>{{company.name}}</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>{{item_value}}</t>
-  </si>
-  <si>
-    <t>{{@barcode invoice_no format=code128 width=180 height=50}}</t>
   </si>
   <si>
     <t>{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}</t>
@@ -96,8 +93,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -217,42 +214,40 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -557,14 +552,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="49.140625" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="5" width="16" style="13" customWidth="1"/>
-    <col min="6" max="6" width="18" style="13" customWidth="1"/>
+    <col min="4" max="5" width="16" style="10" customWidth="1"/>
+    <col min="6" max="6" width="18" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -573,38 +571,36 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="D2" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
+      <c r="B2" s="17"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="16"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7"/>
-      <c r="D3" s="15" t="s">
+      <c r="B3" s="19"/>
+      <c r="D3" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="15"/>
+      <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="D4" s="16" t="s">
+      <c r="B4" s="18"/>
+      <c r="D4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="16"/>
+      <c r="E4" s="12"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -613,13 +609,13 @@
       <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="13" t="s">
         <v>18</v>
       </c>
     </row>
@@ -635,17 +631,17 @@
       <c r="B8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="10" t="e">
+      <c r="C8" s="7" t="e">
         <f>D8/B8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="11" t="e">
+      <c r="F8" s="8" t="e">
         <f>D8+E8</f>
         <v>#VALUE!</v>
       </c>
@@ -656,18 +652,18 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="9">
         <f>SUM(D8:D8)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="9">
         <f>SUM(E8:E8)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="12" t="e">
+      <c r="F10" s="9" t="e">
         <f>SUM(F8:F8)</f>
         <v>#VALUE!</v>
       </c>
@@ -682,7 +678,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -691,17 +687,15 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="D2:F2"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="B12" r:id="rId2"/>
+    <hyperlink ref="B12" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(renderer): remove literal PAGE BREAK text and use invisible CSS page breaks
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$13</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>{{company.name}}</t>
   </si>
@@ -85,15 +86,17 @@
   </si>
   <si>
     <t>{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}</t>
+  </si>
+  <si>
+    <t>{{@barcode 'Invoice No.' + invoice_no + ':Date' + invoice_date format=code128 width=180 height=50}}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.0000_);_(* \(#,##0.0000\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
@@ -194,64 +197,57 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Comma" xfId="2" builtinId="3"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -558,11 +554,12 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="49.140625" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="5" width="16" style="10" customWidth="1"/>
-    <col min="6" max="6" width="18" style="10" customWidth="1"/>
+    <col min="1" max="1" width="39.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="14" style="18" customWidth="1"/>
+    <col min="4" max="4" width="16" style="6" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="18" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -571,51 +568,54 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="D3" s="11" t="s">
+      <c r="B3" s="16"/>
+      <c r="D3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="11"/>
+      <c r="E3" s="7"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="D4" s="12" t="s">
+      <c r="B4" s="17"/>
+      <c r="D4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="12"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="9" t="s">
         <v>18</v>
       </c>
     </row>
@@ -625,23 +625,23 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="7" t="e">
+      <c r="C8" s="21" t="e">
         <f>D8/B8</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="8" t="e">
+      <c r="F8" s="13" t="e">
         <f>D8+E8</f>
         <v>#VALUE!</v>
       </c>
@@ -652,32 +652,27 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="5">
         <f>SUM(D8:D8)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="5">
         <f>SUM(E8:E8)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="9" t="e">
+      <c r="F10" s="5" t="e">
         <f>SUM(F8:F8)</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D11"/>
-      <c r="E11"/>
-      <c r="F11"/>
-    </row>
     <row r="12" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -687,15 +682,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A4:B4"/>
-  </mergeCells>
   <hyperlinks>
     <hyperlink ref="B12" r:id="rId1"/>
+    <hyperlink ref="D2" r:id="rId2" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
   </hyperlinks>
+  <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(renderer): fix merged cells colspan/rowspan inversion and preserve boundary borders
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,8 +15,8 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$13</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$7:$7</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
@@ -97,9 +97,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -151,6 +151,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -201,7 +208,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -210,30 +217,29 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -244,6 +250,12 @@
     </xf>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -551,12 +563,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.85546875" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="14" style="18" customWidth="1"/>
+    <col min="3" max="3" width="14" style="17" customWidth="1"/>
     <col min="4" max="4" width="16" style="6" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" style="6" customWidth="1"/>
     <col min="6" max="6" width="18" style="6" customWidth="1"/>
@@ -567,124 +579,132 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+    </row>
+    <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="15" t="s">
+      <c r="B3" s="13"/>
+      <c r="C3" s="18"/>
+      <c r="F3" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="15"/>
+      <c r="D4" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="16"/>
+      <c r="D5" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E5" s="8"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="20" t="e">
+        <f>D9/B9</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="12" t="e">
+        <f>D9+E9</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="21" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="5">
+        <f>SUM(D9:D9)</f>
         <v>0</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="D3" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="17"/>
-      <c r="D4" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E4" s="8"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="21" t="e">
-        <f>D8/B8</f>
+      <c r="E11" s="5">
+        <f>SUM(E9:E9)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="5" t="e">
+        <f>SUM(F9:F9)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D8" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="13" t="e">
-        <f>D8+E8</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    </row>
+    <row r="13" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C10" s="22" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="5">
-        <f>SUM(D8:D8)</f>
-        <v>0</v>
-      </c>
-      <c r="E10" s="5">
-        <f>SUM(E8:E8)</f>
-        <v>0</v>
-      </c>
-      <c r="F10" s="5" t="e">
-        <f>SUM(F8:F8)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B12" r:id="rId1"/>
-    <hyperlink ref="D2" r:id="rId2" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
+    <hyperlink ref="B13" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(formulas): support arbitrary Excel math, division, running balances, opening_balance, and #DIV/0!
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,18 +15,15 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$14</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$64</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$10:$10</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
-  <si>
-    <t>{{company.name}}</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>Invoice No: {{invoice_no}}</t>
   </si>
@@ -88,7 +85,25 @@
     <t>{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}</t>
   </si>
   <si>
-    <t>{{@barcode 'Invoice No.' + invoice_no + ':Date' + invoice_date format=code128 width=180 height=50}}</t>
+    <t>{{@barcode 'Invoice No.' + invoice_no + ':Date' + invoice_date format=code128 width=180 height=30}}</t>
+  </si>
+  <si>
+    <t>{{#page-footer}}</t>
+  </si>
+  <si>
+    <t>{{/page-footer}}</t>
+  </si>
+  <si>
+    <t>{{#page-header}}</t>
+  </si>
+  <si>
+    <t>{{/page-header}}</t>
+  </si>
+  <si>
+    <t>{{invoices[0].company.name}}</t>
+  </si>
+  <si>
+    <t>{{@page}} of {{@pages}}</t>
   </si>
 </sst>
 </file>
@@ -204,16 +219,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -224,42 +237,48 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="43" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -563,151 +582,255 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="14" style="17" customWidth="1"/>
-    <col min="4" max="4" width="16" style="6" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="18" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="14" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="18" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+    </row>
+    <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A3" s="21" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="23" t="s">
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+    </row>
+    <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+    </row>
+    <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+    </row>
+    <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A6" s="7"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="E6" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="12"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B7" s="10"/>
+      <c r="D7" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-    </row>
-    <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="E7" s="14"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="11"/>
+      <c r="D8" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="15"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="e">
+        <f>D12/B12</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="3" t="e">
+        <f>F11+D12-E12</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C14" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4">
+        <f>SUM(D12:D12)</f>
+        <v>0</v>
+      </c>
+      <c r="E14" s="4">
+        <f>SUM(E12:E12)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="e">
+        <f>SUM(F12:F12)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B19"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+    </row>
+    <row r="21" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="18"/>
-      <c r="F3" s="22" t="s">
+      <c r="B21" s="18"/>
+      <c r="C21" s="17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="15"/>
-      <c r="D4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="D5" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="8"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="20" t="e">
-        <f>D9/B9</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="12" t="e">
-        <f>D9+E9</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C11" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="5">
-        <f>SUM(D9:D9)</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="5">
-        <f>SUM(E9:E9)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="5" t="e">
-        <f>SUM(F9:F9)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="19"/>
+      <c r="B63" s="19"/>
+      <c r="C63" s="19"/>
+      <c r="D63" s="19"/>
+      <c r="E63" s="19"/>
+      <c r="F63" s="19"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
+    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B13" r:id="rId1"/>
-    <hyperlink ref="F3" r:id="rId2" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
+    <hyperlink ref="E6" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
+    <hyperlink ref="C21" r:id="rId2"/>
+    <hyperlink ref="A27" r:id="rId3" display="{{@page}} of {{pages}}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(formatting): fix comma formatting on variable placeholders and inherit directive row borders on footer
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -88,6 +88,9 @@
     <t>{{@barcode 'Invoice No.' + invoice_no + ':Date' + invoice_date format=code128 width=180 height=30}}</t>
   </si>
   <si>
+    <t>This is Footer</t>
+  </si>
+  <si>
     <t>{{#page-footer}}</t>
   </si>
   <si>
@@ -101,9 +104,6 @@
   </si>
   <si>
     <t>{{invoices[0].company.name}}</t>
-  </si>
-  <si>
-    <t>{{@page}} of {{@pages}}</t>
   </si>
 </sst>
 </file>
@@ -195,7 +195,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -218,13 +218,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -266,6 +275,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -273,8 +285,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -595,12 +607,12 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -609,34 +621,34 @@
       <c r="F2" s="13"/>
     </row>
     <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
     </row>
     <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
+        <v>25</v>
+      </c>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
     </row>
     <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
     </row>
     <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A6" s="7"/>
@@ -782,42 +794,48 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="24"/>
+      <c r="C26" s="24"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+    </row>
+    <row r="27" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="19" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
+      <c r="A28" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="19"/>
-      <c r="B63" s="19"/>
-      <c r="C63" s="19"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="19"/>
-      <c r="F63" s="19"/>
+      <c r="A63" s="20"/>
+      <c r="B63" s="20"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D8:E8"/>
@@ -827,10 +845,9 @@
   <hyperlinks>
     <hyperlink ref="E6" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
     <hyperlink ref="C21" r:id="rId2"/>
-    <hyperlink ref="A27" r:id="rId3" display="{{@page}} of {{pages}}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(rendering): eliminate trailing ghost rows preventing extra pages and fix @page/@pages print values
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$64</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$10:$10</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -222,7 +222,7 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="thick">
+      <bottom style="double">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -239,9 +239,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -254,39 +251,42 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -598,11 +598,11 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14" style="5" customWidth="1"/>
-    <col min="4" max="4" width="16" style="5" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="18" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="14" style="4" customWidth="1"/>
+    <col min="4" max="4" width="16" style="4" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="18" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -611,88 +611,88 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
     </row>
     <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
     </row>
     <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
     </row>
     <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
     </row>
     <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A6" s="7"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="E6" s="12" t="s">
+      <c r="A6" s="6"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="E6" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="12"/>
+      <c r="F6" s="22"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="10"/>
-      <c r="D7" s="14" t="s">
+      <c r="B7" s="9"/>
+      <c r="E7" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="E7" s="14"/>
+      <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="D8" s="15" t="s">
+      <c r="B8" s="10"/>
+      <c r="E8" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="15"/>
+      <c r="F8" s="21"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -705,20 +705,20 @@
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="3" t="e">
+      <c r="C12" s="24" t="e">
         <f>D12/B12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="3" t="e">
+      <c r="F12" s="24" t="e">
         <f>F11+D12-E12</f>
         <v>#VALUE!</v>
       </c>
@@ -729,18 +729,18 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="3">
         <f>SUM(D12:D12)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="3">
         <f>SUM(E12:E12)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="4" t="e">
+      <c r="F14" s="3" t="e">
         <f>SUM(F12:F12)</f>
         <v>#VALUE!</v>
       </c>
@@ -781,11 +781,11 @@
       <c r="F19"/>
     </row>
     <row r="21" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="18"/>
-      <c r="C21" s="17" t="s">
+      <c r="B21" s="23"/>
+      <c r="C21" s="12" t="s">
         <v>19</v>
       </c>
     </row>
@@ -795,50 +795,50 @@
       </c>
     </row>
     <row r="26" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="23" t="s">
+      <c r="A26" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
     </row>
     <row r="27" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="13"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="20"/>
-      <c r="B63" s="20"/>
-      <c r="C63" s="20"/>
-      <c r="D63" s="20"/>
-      <c r="E63" s="20"/>
-      <c r="F63" s="20"/>
+      <c r="A63" s="13"/>
+      <c r="B63" s="13"/>
+      <c r="C63" s="13"/>
+      <c r="D63" s="13"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A27:F27"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="A21:B21"/>
   </mergeCells>
@@ -848,6 +848,6 @@
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="69" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(templates): sync SALES_TAX_INV template with page numbering and borders
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$31</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$10:$10</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Invoice No: {{invoice_no}}</t>
   </si>
@@ -86,9 +86,6 @@
   </si>
   <si>
     <t>{{@barcode 'Invoice No.' + invoice_no + ':Date' + invoice_date format=code128 width=180 height=30}}</t>
-  </si>
-  <si>
-    <t>This is Footer</t>
   </si>
   <si>
     <t>{{#page-footer}}</t>
@@ -233,7 +230,7 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -264,9 +261,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -594,7 +588,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F63"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="39.85546875" customWidth="1"/>
@@ -607,18 +601,18 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="A2" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
     </row>
     <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A3" s="17" t="s">
@@ -632,7 +626,7 @@
     </row>
     <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B4" s="14"/>
       <c r="C4" s="14"/>
@@ -654,27 +648,27 @@
       <c r="A6" s="6"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="22"/>
+      <c r="F6" s="21"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B7" s="9"/>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="20"/>
+      <c r="F7" s="19"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>1</v>
       </c>
       <c r="B8" s="10"/>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="21"/>
+      <c r="F8" s="20"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -705,20 +699,20 @@
       <c r="A12" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="24" t="s">
+      <c r="B12" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="24" t="e">
+      <c r="C12" s="23" t="e">
         <f>D12/B12</f>
         <v>#VALUE!</v>
       </c>
-      <c r="D12" s="24" t="s">
+      <c r="D12" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="24" t="e">
+      <c r="F12" s="23" t="e">
         <f>F11+D12-E12</f>
         <v>#VALUE!</v>
       </c>
@@ -781,10 +775,10 @@
       <c r="F19"/>
     </row>
     <row r="21" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="23"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="12" t="s">
         <v>19</v>
       </c>
@@ -794,48 +788,45 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="s">
+    <row r="29" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+    </row>
+    <row r="30" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="13"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-    </row>
-    <row r="27" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="18"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="13"/>
-      <c r="B63" s="13"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="13"/>
-      <c r="E63" s="13"/>
-      <c r="F63" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="13"/>
+      <c r="B66" s="13"/>
+      <c r="C66" s="13"/>
+      <c r="D66" s="13"/>
+      <c r="E66" s="13"/>
+      <c r="F66" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="E8:F8"/>

</xml_diff>

<commit_message>
feat(engine): add {{#repeat-on-page}} tag for repeating table header rows across pages
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,15 +15,15 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$1:$F$31</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$10:$10</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$2:$F$35</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$12:$12</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>Invoice No: {{invoice_no}}</t>
   </si>
@@ -101,6 +101,18 @@
   </si>
   <si>
     <t>{{invoices[0].company.name}}</t>
+  </si>
+  <si>
+    <t>Authorized By</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>Total Value</t>
+  </si>
+  <si>
+    <t>Total ST.</t>
   </si>
 </sst>
 </file>
@@ -111,7 +123,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,13 +178,27 @@
     </font>
     <font>
       <b/>
-      <sz val="22"/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,8 +217,14 @@
         <bgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -218,8 +250,23 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -230,7 +277,7 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -258,27 +305,37 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -588,170 +645,156 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A2:G70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.85546875" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14" style="4" customWidth="1"/>
-    <col min="4" max="4" width="16" style="4" customWidth="1"/>
-    <col min="5" max="5" width="18.5703125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="18" style="4" customWidth="1"/>
+    <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="14" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="18" t="s">
+    <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A4" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-    </row>
-    <row r="3" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="17" t="s">
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+    </row>
+    <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-    </row>
-    <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+    </row>
+    <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-    </row>
-    <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-    </row>
-    <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A6" s="6"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="E6" s="21" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A8" s="6"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="E8" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="21"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="9"/>
-      <c r="E7" s="19" t="s">
+      <c r="F8" s="19"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B9" s="9"/>
+      <c r="E9" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="F7" s="19"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="F9" s="17"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="E8" s="20" t="s">
+      <c r="B10" s="10"/>
+      <c r="E10" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="20"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="F10" s="18"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="23" t="e">
-        <f>D12/B12</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>18</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" s="23" t="e">
-        <f>F11+D12-E12</f>
-        <v>#VALUE!</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="15" t="e">
+        <f>D14/B14</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="15" t="e">
+        <f>F13+D14-E14</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C14" s="11" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C16" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D14" s="3">
-        <f>SUM(D12:D12)</f>
+      <c r="D16" s="3">
+        <f>SUM(D14:D14)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="3">
-        <f>SUM(E12:E12)</f>
+      <c r="E16" s="3">
+        <f>SUM(E14:E14)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="3" t="e">
-        <f>SUM(F12:F12)</f>
+      <c r="F16" s="3" t="e">
+        <f>SUM(F14:F14)</f>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B15"/>
-      <c r="C15"/>
-      <c r="D15"/>
-      <c r="E15"/>
-      <c r="F15"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B16"/>
-      <c r="C16"/>
-      <c r="D16"/>
-      <c r="E16"/>
-      <c r="F16"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B17"/>
@@ -761,84 +804,145 @@
       <c r="F17"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B18"/>
-      <c r="C18"/>
       <c r="D18"/>
-      <c r="E18"/>
+      <c r="E18" s="25" t="s">
+        <v>27</v>
+      </c>
       <c r="F18"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B19"/>
-      <c r="C19"/>
       <c r="D19"/>
-      <c r="E19"/>
-      <c r="F19"/>
-    </row>
-    <row r="21" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="E19" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="27">
+        <f>SUM(D14:D14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20" s="27">
+        <f>SUM(E14:E14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B21"/>
+      <c r="C21"/>
+      <c r="D21"/>
+      <c r="E21" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="27" t="e">
+        <f>SUM(F14:F14)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B22"/>
+      <c r="C22"/>
+      <c r="D22"/>
+    </row>
+    <row r="23" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="22"/>
-      <c r="C21" s="12" t="s">
+      <c r="B23" s="20"/>
+      <c r="C23" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="28" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="23" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="15" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>21</v>
       </c>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-    </row>
-    <row r="30" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13"/>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13"/>
-      <c r="F30" s="13"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="B32"/>
+      <c r="C32"/>
+      <c r="D32"/>
+      <c r="E32"/>
+      <c r="F32"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B33"/>
+      <c r="C33"/>
+      <c r="D33"/>
+      <c r="E33"/>
+      <c r="F33"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="21"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="13"/>
-      <c r="B66" s="13"/>
-      <c r="C66" s="13"/>
-      <c r="D66" s="13"/>
-      <c r="E66" s="13"/>
-      <c r="F66" s="13"/>
+      <c r="B35"/>
+      <c r="C35"/>
+      <c r="D35"/>
+      <c r="E35"/>
+      <c r="F35"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B36"/>
+      <c r="C36"/>
+      <c r="D36"/>
+      <c r="E36"/>
+      <c r="F36"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B37"/>
+      <c r="C37"/>
+      <c r="D37"/>
+      <c r="E37"/>
+      <c r="F37"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="13"/>
+      <c r="B70" s="13"/>
+      <c r="C70" s="13"/>
+      <c r="D70" s="13"/>
+      <c r="E70" s="13"/>
+      <c r="F70" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E9:F9"/>
+    <mergeCell ref="E10:F10"/>
     <mergeCell ref="E8:F8"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="A21:B21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E6" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
-    <hyperlink ref="C21" r:id="rId2"/>
+    <hyperlink ref="E8" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
+    <hyperlink ref="C23" r:id="rId2"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="73" orientation="portrait" r:id="rId3"/>
+  <pageSetup paperSize="9" scale="88" orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(studio): recreate studio in modern white theme using Tailwind CSS, PostCSS, and clean SVG icons
</commit_message>
<xml_diff>
--- a/templates/SALES_TAX_INV.xlsx
+++ b/templates/SALES_TAX_INV.xlsx
@@ -15,15 +15,15 @@
     <sheet name="Invoice" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$2:$F$35</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$12:$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Invoice!$A$2:$F$37</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">Invoice!$13:$13</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
   <si>
     <t>Invoice No: {{invoice_no}}</t>
   </si>
@@ -113,6 +113,12 @@
   </si>
   <si>
     <t>Total ST.</t>
+  </si>
+  <si>
+    <t>{{#repeat-header}}</t>
+  </si>
+  <si>
+    <t>{{/repeat-header}}</t>
   </si>
 </sst>
 </file>
@@ -184,15 +190,15 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
+      <sz val="8"/>
+      <color theme="3" tint="0.39997558519241921"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -277,7 +283,7 @@
     <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -305,6 +311,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -331,13 +340,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -645,7 +654,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:G70"/>
+  <dimension ref="A2:G72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -662,24 +671,24 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
     </row>
     <row r="5" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="16"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
     </row>
     <row r="6" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
@@ -702,204 +711,205 @@
       <c r="F7" s="14"/>
     </row>
     <row r="8" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A8" s="6"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="E8" s="19" t="s">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+    </row>
+    <row r="9" spans="1:6" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A9" s="6"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="E9" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="19"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="9"/>
-      <c r="E9" s="17" t="s">
+      <c r="F9" s="20"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B10" s="9"/>
+      <c r="E10" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="F9" s="17"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="F10" s="18"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="E10" s="18" t="s">
+      <c r="B11" s="10"/>
+      <c r="E11" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="F10" s="18"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="F11" s="19"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F13" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="15" t="e">
-        <f>D14/B14</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="F14" s="15" t="e">
-        <f>F13+D14-E14</f>
-        <v>#VALUE!</v>
-      </c>
+      <c r="A14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="16" t="e">
+        <f>D16/B16</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="D16" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="16" t="e">
+        <f>F15+D16-E16</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C16" s="11" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C18" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="3">
-        <f>SUM(D14:D14)</f>
+      <c r="D18" s="3">
+        <f>SUM(D16:D16)</f>
         <v>0</v>
       </c>
-      <c r="E16" s="3">
-        <f>SUM(E14:E14)</f>
+      <c r="E18" s="3">
+        <f>SUM(E16:E16)</f>
         <v>0</v>
       </c>
-      <c r="F16" s="3" t="e">
-        <f>SUM(F14:F14)</f>
+      <c r="F18" s="3" t="e">
+        <f>SUM(F16:F16)</f>
         <v>#VALUE!</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B17"/>
-      <c r="C17"/>
-      <c r="D17"/>
-      <c r="E17"/>
-      <c r="F17"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D18"/>
-      <c r="E18" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F18"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B19"/>
+      <c r="C19"/>
       <c r="D19"/>
-      <c r="E19" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="27">
-        <f>SUM(D14:D14)</f>
-        <v>0</v>
-      </c>
+      <c r="E19"/>
+      <c r="F19"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B20"/>
-      <c r="C20"/>
       <c r="D20"/>
-      <c r="E20" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="F20" s="27">
-        <f>SUM(E14:E14)</f>
-        <v>0</v>
-      </c>
+      <c r="E20" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B21"/>
-      <c r="C21"/>
       <c r="D21"/>
-      <c r="E21" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="27" t="e">
-        <f>SUM(F14:F14)</f>
-        <v>#VALUE!</v>
+      <c r="E21" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="27">
+        <f>SUM(D16:D16)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22"/>
-    </row>
-    <row r="23" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="20" t="s">
+      <c r="E22" s="25" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22" s="27">
+        <f>SUM(E16:E16)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B23"/>
+      <c r="C23"/>
+      <c r="D23"/>
+      <c r="E23" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="27" t="e">
+        <f>SUM(F16:F16)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B24"/>
+      <c r="C24"/>
+      <c r="D24"/>
+    </row>
+    <row r="25" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="12" t="s">
+      <c r="B25" s="21"/>
+      <c r="C25" s="12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="23" t="s">
+    <row r="30" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="24" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>21</v>
       </c>
-      <c r="B32"/>
-      <c r="C32"/>
-      <c r="D32"/>
-      <c r="E32"/>
-      <c r="F32"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B33"/>
-      <c r="C33"/>
-      <c r="D33"/>
-      <c r="E33"/>
-      <c r="F33"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
+      <c r="B34"/>
+      <c r="C34"/>
+      <c r="D34"/>
+      <c r="E34"/>
+      <c r="F34"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>22</v>
-      </c>
       <c r="B35"/>
       <c r="C35"/>
       <c r="D35"/>
@@ -907,39 +917,58 @@
       <c r="F35"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B36"/>
-      <c r="C36"/>
-      <c r="D36"/>
-      <c r="E36"/>
-      <c r="F36"/>
+      <c r="A36" s="22"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="22"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>22</v>
+      </c>
       <c r="B37"/>
       <c r="C37"/>
       <c r="D37"/>
       <c r="E37"/>
       <c r="F37"/>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="13"/>
-      <c r="B70" s="13"/>
-      <c r="C70" s="13"/>
-      <c r="D70" s="13"/>
-      <c r="E70" s="13"/>
-      <c r="F70" s="13"/>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B38"/>
+      <c r="C38"/>
+      <c r="D38"/>
+      <c r="E38"/>
+      <c r="F38"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B39"/>
+      <c r="C39"/>
+      <c r="D39"/>
+      <c r="E39"/>
+      <c r="F39"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="13"/>
+      <c r="B72" s="13"/>
+      <c r="C72" s="13"/>
+      <c r="D72" s="13"/>
+      <c r="E72" s="13"/>
+      <c r="F72" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A25:B25"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="E9:F9"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="E8:F8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
-    <hyperlink ref="C23" r:id="rId2"/>
+    <hyperlink ref="E9" r:id="rId1" display="{{@qr 'Invoice No.' + invoice_no + ':Date' + invoice_date width=90 height=90}}"/>
+    <hyperlink ref="C25" r:id="rId2"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>